<commit_message>
updated the model comparison
</commit_message>
<xml_diff>
--- a/Model_comparison.xlsx
+++ b/Model_comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Large_Projects\infosys_project_1\CreditPathAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B747256-114F-4D0C-98CE-96F1211B44B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77B77DAF-88CD-433A-A9A7-38A61BC4D9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset1_File1" sheetId="1" r:id="rId1"/>
@@ -60,9 +60,6 @@
     <t>CV Mean</t>
   </si>
   <si>
-    <t>Default (unknown)</t>
-  </si>
-  <si>
     <t>KNN (n=10)</t>
   </si>
   <si>
@@ -85,6 +82,9 @@
   </si>
   <si>
     <t xml:space="preserve">F1-score </t>
+  </si>
+  <si>
+    <t>GaussianNB</t>
   </si>
 </sst>
 </file>
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -155,6 +155,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -391,13 +394,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -1578,174 +1581,174 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2">
-        <v>0.99919999999999998</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.99929999999999997</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0.99970000000000003</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2">
-        <v>1</v>
+        <v>0.88370000000000004</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0.88270000000000004</v>
+      </c>
+      <c r="D2">
+        <v>0.95140000000000002</v>
+      </c>
+      <c r="E2">
+        <v>0.84</v>
+      </c>
+      <c r="F2">
+        <v>0.85</v>
+      </c>
+      <c r="G2">
+        <v>0.84</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="2">
-        <v>0.90780000000000005</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.90849999999999997</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.96479999999999999</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0.89</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0.89</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0.89</v>
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>0.8669</v>
+      </c>
+      <c r="C3">
+        <v>0.86809999999999998</v>
+      </c>
+      <c r="D3">
+        <v>0.90029999999999999</v>
+      </c>
+      <c r="E3">
+        <v>0.78</v>
+      </c>
+      <c r="F3">
+        <v>0.85</v>
+      </c>
+      <c r="G3">
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
-        <v>0.74660000000000004</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.75119999999999998</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.7571</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0.61</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0.69</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.62</v>
+      <c r="B4">
+        <v>0.76539999999999997</v>
+      </c>
+      <c r="C4">
+        <v>0.76759999999999995</v>
+      </c>
+      <c r="D4">
+        <v>0.71220000000000006</v>
+      </c>
+      <c r="E4">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="F4">
+        <v>0.7</v>
+      </c>
+      <c r="G4">
+        <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2">
-        <v>0.99950000000000006</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.99980000000000002</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.99939999999999996</v>
-      </c>
-      <c r="E5" s="2">
-        <v>1</v>
-      </c>
-      <c r="F5" s="2">
-        <v>1</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0.91069999999999995</v>
+      </c>
+      <c r="C5">
+        <v>0.91279999999999994</v>
+      </c>
+      <c r="D5">
+        <v>0.88119999999999998</v>
+      </c>
+      <c r="E5">
+        <v>0.88</v>
+      </c>
+      <c r="F5">
+        <v>0.88</v>
+      </c>
+      <c r="G5">
+        <v>0.88</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
-        <v>0.99990000000000001</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.99990000000000001</v>
-      </c>
-      <c r="D6" s="2">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2">
-        <v>1</v>
-      </c>
-      <c r="F6" s="2">
-        <v>1</v>
-      </c>
-      <c r="G6" s="2">
-        <v>1</v>
+      <c r="B6">
+        <v>0.92930000000000001</v>
+      </c>
+      <c r="C6">
+        <v>0.93230000000000002</v>
+      </c>
+      <c r="D6">
+        <v>0.98319999999999996</v>
+      </c>
+      <c r="E6">
+        <v>0.9</v>
+      </c>
+      <c r="F6">
+        <v>0.91</v>
+      </c>
+      <c r="G6">
+        <v>0.91</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.99990000000000001</v>
-      </c>
-      <c r="D7" s="2">
-        <v>1</v>
-      </c>
-      <c r="E7" s="2">
-        <v>1</v>
-      </c>
-      <c r="F7" s="2">
-        <v>1</v>
-      </c>
-      <c r="G7" s="2">
-        <v>1</v>
+      <c r="B7">
+        <v>0.93120000000000003</v>
+      </c>
+      <c r="C7">
+        <v>0.93289999999999995</v>
+      </c>
+      <c r="D7">
+        <v>0.98419999999999996</v>
+      </c>
+      <c r="E7">
+        <v>0.91</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.91</v>
+      </c>
+      <c r="G7">
+        <v>0.91</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="2">
-        <v>0.9012</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0.90229999999999999</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0.96719999999999995</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0.89</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0.87</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0.88</v>
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>0.81740000000000002</v>
+      </c>
+      <c r="C8">
+        <v>0.81850000000000001</v>
+      </c>
+      <c r="D8">
+        <v>0.87080000000000002</v>
+      </c>
+      <c r="E8">
+        <v>0.75</v>
+      </c>
+      <c r="F8">
+        <v>0.76</v>
+      </c>
+      <c r="G8">
+        <v>0.75</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2756,13 +2759,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>

</xml_diff>